<commit_message>
AIN data gap fix: backfill Aug13-16 + staleness guard
Bug: build_case chạy 17/08 trên scratch CSV fetch 13/08 → thiếu
Aug13-16 (5 ngày). Không có guard → build câm.

Fix:
- Re-fetch AIN klines Aug13-16, OI, funding (1368 entries), LSR
- Schema fix: perp CSV dùng open/close/ret_1d%, OI dùng oi_usd/oi_token
- Rebuild CASE_AIN.xlsx: 228 rows Jan01-Aug16, validate PASS
- build_case.py: thêm STALENESS GUARD (gap > 2d → RuntimeError)
- Lesson L-BUG-STALE-CASE ghi vào CASE_INDEX LESSONS

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_AIN.xlsx
+++ b/docs/case_files/CASE_AIN.xlsx
@@ -635,7 +635,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>fullyDelisted=False, offsell=False, offline=False</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX226"/>
+  <dimension ref="A1:AX230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29029,32 +29029,16 @@
       <c r="U201" s="14" t="n">
         <v>0.84</v>
       </c>
-      <c r="V201" s="14" t="n">
-        <v>0.6909999999999999</v>
-      </c>
-      <c r="W201" s="14" t="n">
-        <v>0.7282999999999999</v>
-      </c>
-      <c r="X201" s="14" t="n">
-        <v>1.7173</v>
-      </c>
-      <c r="Y201" s="14" t="n">
-        <v>6.04</v>
-      </c>
-      <c r="Z201" s="14" t="n">
-        <v>25.46</v>
-      </c>
-      <c r="AA201" s="14" t="n">
-        <v>1.7394</v>
-      </c>
-      <c r="AB201" s="14" t="n">
-        <v>2.5174</v>
-      </c>
-      <c r="AC201" s="14" t="n">
-        <v>2.962</v>
-      </c>
+      <c r="V201" s="14" t="inlineStr"/>
+      <c r="W201" s="14" t="inlineStr"/>
+      <c r="X201" s="14" t="inlineStr"/>
+      <c r="Y201" s="14" t="inlineStr"/>
+      <c r="Z201" s="14" t="inlineStr"/>
+      <c r="AA201" s="14" t="inlineStr"/>
+      <c r="AB201" s="14" t="inlineStr"/>
+      <c r="AC201" s="14" t="inlineStr"/>
       <c r="AD201" s="14" t="n">
-        <v>1.060936494003794</v>
+        <v>1.0609</v>
       </c>
       <c r="AE201" s="14" t="inlineStr"/>
       <c r="AF201" s="14" t="inlineStr"/>
@@ -29093,7 +29077,7 @@
       </c>
       <c r="AP201" s="14" t="inlineStr">
         <is>
-          <t>freshwatch</t>
+          <t>fapi_LSR_30d</t>
         </is>
       </c>
       <c r="AQ201" s="14" t="inlineStr"/>
@@ -29192,9 +29176,7 @@
       <c r="V202" s="14" t="n">
         <v>0.6479</v>
       </c>
-      <c r="W202" s="14" t="n">
-        <v>0.6875</v>
-      </c>
+      <c r="W202" s="14" t="inlineStr"/>
       <c r="X202" s="14" t="n">
         <v>1.5279</v>
       </c>
@@ -29352,9 +29334,7 @@
       <c r="V203" s="14" t="n">
         <v>0.6830000000000001</v>
       </c>
-      <c r="W203" s="14" t="n">
-        <v>0.6735</v>
-      </c>
+      <c r="W203" s="14" t="inlineStr"/>
       <c r="X203" s="14" t="n">
         <v>1.4827</v>
       </c>
@@ -29518,12 +29498,8 @@
       <c r="X204" s="14" t="n">
         <v>1.1298</v>
       </c>
-      <c r="Y204" s="14" t="n">
-        <v>4.97</v>
-      </c>
-      <c r="Z204" s="14" t="n">
-        <v>-12.16</v>
-      </c>
+      <c r="Y204" s="14" t="inlineStr"/>
+      <c r="Z204" s="14" t="inlineStr"/>
       <c r="AA204" s="14" t="n">
         <v>1.8258</v>
       </c>
@@ -29835,9 +29811,7 @@
       <c r="W206" s="14" t="n">
         <v>0.8042</v>
       </c>
-      <c r="X206" s="14" t="n">
-        <v>1.0254</v>
-      </c>
+      <c r="X206" s="14" t="inlineStr"/>
       <c r="Y206" s="14" t="n">
         <v>-0.09</v>
       </c>
@@ -33196,6 +33170,662 @@
         </is>
       </c>
       <c r="AX226" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B227" s="14" t="n">
+        <v>0.07975333</v>
+      </c>
+      <c r="C227" s="14" t="n">
+        <v>0.07552</v>
+      </c>
+      <c r="D227" s="14" t="n">
+        <v>0.08304</v>
+      </c>
+      <c r="E227" s="14" t="n">
+        <v>0.07547</v>
+      </c>
+      <c r="F227" s="14" t="n">
+        <v>0.08075</v>
+      </c>
+      <c r="G227" s="14" t="n">
+        <v>1966798.95</v>
+      </c>
+      <c r="H227" s="14" t="n">
+        <v>49.7654</v>
+      </c>
+      <c r="I227" s="14" t="n">
+        <v>0.00023565</v>
+      </c>
+      <c r="J227" s="14" t="n">
+        <v>0.00013208</v>
+      </c>
+      <c r="K227" s="14" t="n">
+        <v>0.00033884</v>
+      </c>
+      <c r="L227" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="M227" s="14" t="n">
+        <v>4415138.27166272</v>
+      </c>
+      <c r="N227" s="14" t="n">
+        <v>58494016</v>
+      </c>
+      <c r="O227" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="P227" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q227" s="14" t="n">
+        <v>6.93947821</v>
+      </c>
+      <c r="R227" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S227" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="T227" s="14" t="n">
+        <v>1.071</v>
+      </c>
+      <c r="U227" s="14" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="V227" s="14" t="n">
+        <v>0.7219</v>
+      </c>
+      <c r="W227" s="14" t="n">
+        <v>0.7135</v>
+      </c>
+      <c r="X227" s="14" t="n">
+        <v>0.7461</v>
+      </c>
+      <c r="Y227" s="14" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="Z227" s="14" t="n">
+        <v>-2.33</v>
+      </c>
+      <c r="AA227" s="14" t="n">
+        <v>1.4657</v>
+      </c>
+      <c r="AB227" s="14" t="n">
+        <v>2.0303</v>
+      </c>
+      <c r="AC227" s="14" t="n">
+        <v>2.3003</v>
+      </c>
+      <c r="AD227" s="14" t="n">
+        <v>0.9887</v>
+      </c>
+      <c r="AE227" s="14" t="inlineStr"/>
+      <c r="AF227" s="14" t="inlineStr"/>
+      <c r="AG227" s="14" t="inlineStr"/>
+      <c r="AH227" s="14" t="inlineStr"/>
+      <c r="AI227" s="14" t="inlineStr">
+        <is>
+          <t>alpha_klines_store(forward_2026-08-04,venue=binance_alpha)</t>
+        </is>
+      </c>
+      <c r="AJ227" s="14" t="inlineStr">
+        <is>
+          <t>ABSTAIN(bapi_klines9==klines5_L48)</t>
+        </is>
+      </c>
+      <c r="AK227" s="14" t="inlineStr">
+        <is>
+          <t>ABSTAIN(Nansen_LOCKED)</t>
+        </is>
+      </c>
+      <c r="AL227" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AM227" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AN227" s="14" t="inlineStr"/>
+      <c r="AO227" s="14" t="inlineStr">
+        <is>
+          <t>fapi_klines_1d</t>
+        </is>
+      </c>
+      <c r="AP227" s="14" t="inlineStr">
+        <is>
+          <t>fapi_LSR_30d</t>
+        </is>
+      </c>
+      <c r="AQ227" s="14" t="n">
+        <v>0.6792</v>
+      </c>
+      <c r="AR227" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AS227" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AT227" s="14" t="inlineStr"/>
+      <c r="AU227" s="14" t="inlineStr"/>
+      <c r="AV227" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AW227" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AX227" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B228" s="14" t="n">
+        <v>0.07756</v>
+      </c>
+      <c r="C228" s="14" t="n">
+        <v>0.08074000000000001</v>
+      </c>
+      <c r="D228" s="14" t="n">
+        <v>0.08248999999999999</v>
+      </c>
+      <c r="E228" s="14" t="n">
+        <v>0.07156</v>
+      </c>
+      <c r="F228" s="14" t="n">
+        <v>0.07863000000000001</v>
+      </c>
+      <c r="G228" s="14" t="n">
+        <v>2676664.8</v>
+      </c>
+      <c r="H228" s="14" t="n">
+        <v>47.1293</v>
+      </c>
+      <c r="I228" s="14" t="n">
+        <v>0.00023788</v>
+      </c>
+      <c r="J228" s="14" t="n">
+        <v>0.00011413</v>
+      </c>
+      <c r="K228" s="14" t="n">
+        <v>0.00033701</v>
+      </c>
+      <c r="L228" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="M228" s="14" t="n">
+        <v>4747108.96337924</v>
+      </c>
+      <c r="N228" s="14" t="n">
+        <v>58789853</v>
+      </c>
+      <c r="O228" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="P228" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q228" s="14" t="n">
+        <v>-2.625387</v>
+      </c>
+      <c r="R228" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S228" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="T228" s="14" t="n">
+        <v>1.151</v>
+      </c>
+      <c r="U228" s="14" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="V228" s="14" t="n">
+        <v>0.7565</v>
+      </c>
+      <c r="W228" s="14" t="n">
+        <v>0.7429</v>
+      </c>
+      <c r="X228" s="14" t="n">
+        <v>0.7441</v>
+      </c>
+      <c r="Y228" s="14" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="Z228" s="14" t="n">
+        <v>-9.93</v>
+      </c>
+      <c r="AA228" s="14" t="n">
+        <v>1.4803</v>
+      </c>
+      <c r="AB228" s="14" t="n">
+        <v>1.9568</v>
+      </c>
+      <c r="AC228" s="14" t="n">
+        <v>2.1211</v>
+      </c>
+      <c r="AD228" s="14" t="n">
+        <v>0.8907</v>
+      </c>
+      <c r="AE228" s="14" t="inlineStr"/>
+      <c r="AF228" s="14" t="inlineStr"/>
+      <c r="AG228" s="14" t="inlineStr"/>
+      <c r="AH228" s="14" t="inlineStr"/>
+      <c r="AI228" s="14" t="inlineStr">
+        <is>
+          <t>alpha_klines_store(forward_2026-08-04,venue=binance_alpha)</t>
+        </is>
+      </c>
+      <c r="AJ228" s="14" t="inlineStr">
+        <is>
+          <t>ABSTAIN(bapi_klines9==klines5_L48)</t>
+        </is>
+      </c>
+      <c r="AK228" s="14" t="inlineStr">
+        <is>
+          <t>ABSTAIN(Nansen_LOCKED)</t>
+        </is>
+      </c>
+      <c r="AL228" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AM228" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AN228" s="14" t="inlineStr"/>
+      <c r="AO228" s="14" t="inlineStr">
+        <is>
+          <t>fapi_klines_1d</t>
+        </is>
+      </c>
+      <c r="AP228" s="14" t="inlineStr">
+        <is>
+          <t>fapi_LSR_30d</t>
+        </is>
+      </c>
+      <c r="AQ228" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR228" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AS228" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AT228" s="14" t="inlineStr"/>
+      <c r="AU228" s="14" t="inlineStr"/>
+      <c r="AV228" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AW228" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AX228" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B229" s="14" t="n">
+        <v>0.08093333</v>
+      </c>
+      <c r="C229" s="14" t="n">
+        <v>0.07863000000000001</v>
+      </c>
+      <c r="D229" s="14" t="n">
+        <v>0.08484999999999999</v>
+      </c>
+      <c r="E229" s="14" t="n">
+        <v>0.07847</v>
+      </c>
+      <c r="F229" s="14" t="n">
+        <v>0.07948</v>
+      </c>
+      <c r="G229" s="14" t="n">
+        <v>1562930.93</v>
+      </c>
+      <c r="H229" s="14" t="n">
+        <v>46.5553</v>
+      </c>
+      <c r="I229" s="14" t="n">
+        <v>0.00014031</v>
+      </c>
+      <c r="J229" s="14" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="K229" s="14" t="n">
+        <v>0.00024132</v>
+      </c>
+      <c r="L229" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="M229" s="14" t="n">
+        <v>4724816.62668</v>
+      </c>
+      <c r="N229" s="14" t="n">
+        <v>60089236</v>
+      </c>
+      <c r="O229" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="P229" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q229" s="14" t="n">
+        <v>1.08101234</v>
+      </c>
+      <c r="R229" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S229" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="T229" s="14" t="n">
+        <v>1.146</v>
+      </c>
+      <c r="U229" s="14" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="V229" s="14" t="n">
+        <v>0.5780999999999999</v>
+      </c>
+      <c r="W229" s="14" t="n">
+        <v>0.6764</v>
+      </c>
+      <c r="X229" s="14" t="n">
+        <v>1.0743</v>
+      </c>
+      <c r="Y229" s="14" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="Z229" s="14" t="n">
+        <v>31.17</v>
+      </c>
+      <c r="AA229" s="14" t="n">
+        <v>1.4668</v>
+      </c>
+      <c r="AB229" s="14" t="n">
+        <v>2.5373</v>
+      </c>
+      <c r="AC229" s="14" t="n">
+        <v>2.6023</v>
+      </c>
+      <c r="AD229" s="14" t="n">
+        <v>0.8709</v>
+      </c>
+      <c r="AE229" s="14" t="inlineStr"/>
+      <c r="AF229" s="14" t="inlineStr"/>
+      <c r="AG229" s="14" t="inlineStr"/>
+      <c r="AH229" s="14" t="inlineStr"/>
+      <c r="AI229" s="14" t="inlineStr">
+        <is>
+          <t>alpha_klines_store(forward_2026-08-04,venue=binance_alpha)</t>
+        </is>
+      </c>
+      <c r="AJ229" s="14" t="inlineStr">
+        <is>
+          <t>ABSTAIN(bapi_klines9==klines5_L48)</t>
+        </is>
+      </c>
+      <c r="AK229" s="14" t="inlineStr">
+        <is>
+          <t>ABSTAIN(Nansen_LOCKED)</t>
+        </is>
+      </c>
+      <c r="AL229" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AM229" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AN229" s="14" t="inlineStr"/>
+      <c r="AO229" s="14" t="inlineStr">
+        <is>
+          <t>fapi_klines_1d</t>
+        </is>
+      </c>
+      <c r="AP229" s="14" t="inlineStr">
+        <is>
+          <t>fapi_LSR_30d</t>
+        </is>
+      </c>
+      <c r="AQ229" s="14" t="n">
+        <v>0.9758</v>
+      </c>
+      <c r="AR229" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AS229" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AT229" s="14" t="inlineStr"/>
+      <c r="AU229" s="14" t="inlineStr"/>
+      <c r="AV229" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AW229" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AX229" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B230" s="14" t="n">
+        <v>0.07915</v>
+      </c>
+      <c r="C230" s="14" t="n">
+        <v>0.07947</v>
+      </c>
+      <c r="D230" s="14" t="n">
+        <v>0.08115</v>
+      </c>
+      <c r="E230" s="14" t="n">
+        <v>0.07772</v>
+      </c>
+      <c r="F230" s="14" t="n">
+        <v>0.07858</v>
+      </c>
+      <c r="G230" s="14" t="n">
+        <v>1013262.6</v>
+      </c>
+      <c r="H230" s="14" t="n">
+        <v>45.4095</v>
+      </c>
+      <c r="I230" s="14" t="n">
+        <v>0.00012424</v>
+      </c>
+      <c r="J230" s="14" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="K230" s="14" t="n">
+        <v>0.00027931</v>
+      </c>
+      <c r="L230" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="M230" s="14" t="n">
+        <v>4786107.58482</v>
+      </c>
+      <c r="N230" s="14" t="n">
+        <v>60232917</v>
+      </c>
+      <c r="O230" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="P230" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q230" s="14" t="n">
+        <v>-1.13236034</v>
+      </c>
+      <c r="R230" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S230" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="T230" s="14" t="n">
+        <v>1.153</v>
+      </c>
+      <c r="U230" s="14" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="V230" s="14" t="n">
+        <v>0.5469000000000001</v>
+      </c>
+      <c r="W230" s="14" t="n">
+        <v>0.6161</v>
+      </c>
+      <c r="X230" s="14" t="n">
+        <v>1.0802</v>
+      </c>
+      <c r="Y230" s="14" t="n">
+        <v>-3.62</v>
+      </c>
+      <c r="Z230" s="14" t="n">
+        <v>27.22</v>
+      </c>
+      <c r="AA230" s="14" t="n">
+        <v>1.4127</v>
+      </c>
+      <c r="AB230" s="14" t="n">
+        <v>2.5829</v>
+      </c>
+      <c r="AC230" s="14" t="n">
+        <v>2.7679</v>
+      </c>
+      <c r="AD230" s="14" t="n">
+        <v>0.8319</v>
+      </c>
+      <c r="AE230" s="14" t="inlineStr"/>
+      <c r="AF230" s="14" t="inlineStr"/>
+      <c r="AG230" s="14" t="inlineStr"/>
+      <c r="AH230" s="14" t="inlineStr"/>
+      <c r="AI230" s="14" t="inlineStr">
+        <is>
+          <t>alpha_klines_store(forward_2026-08-04,venue=binance_alpha)</t>
+        </is>
+      </c>
+      <c r="AJ230" s="14" t="inlineStr">
+        <is>
+          <t>ABSTAIN(bapi_klines9==klines5_L48)</t>
+        </is>
+      </c>
+      <c r="AK230" s="14" t="inlineStr">
+        <is>
+          <t>ABSTAIN(Nansen_LOCKED)</t>
+        </is>
+      </c>
+      <c r="AL230" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AM230" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AN230" s="14" t="inlineStr"/>
+      <c r="AO230" s="14" t="inlineStr">
+        <is>
+          <t>fapi_klines_1d</t>
+        </is>
+      </c>
+      <c r="AP230" s="14" t="inlineStr">
+        <is>
+          <t>fapi_LSR_30d</t>
+        </is>
+      </c>
+      <c r="AQ230" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR230" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AS230" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AT230" s="14" t="inlineStr"/>
+      <c r="AU230" s="14" t="inlineStr"/>
+      <c r="AV230" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AW230" s="14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AX230" s="14" t="inlineStr">
         <is>
           <t>false</t>
         </is>

</xml_diff>

<commit_message>
GUA+APR rebuild Aug10-16 + spot cols filled; AIN spot patch applied
- GUA: perp Aug10-16 appended (238r), funding +33, OI+LSR fresh 30d
- APR: perp Aug10-16 appended (298r), funding +36, OI+LSR fresh 30d
- GUA/APR: LSR pos_r = null (fapi data absent for both — A-0b known gap)
- Spot cols (31-33) re-filled: GUA 47r (Aug16), APR 47r (Aug16), AIN 47r (Aug16)
- AIN spot patch (from temp) applied after Excel lock resolved

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_AIN.xlsx
+++ b/docs/case_files/CASE_AIN.xlsx
@@ -26388,9 +26388,11 @@
       <c r="AD184" s="14" t="n">
         <v>1.036320722045512</v>
       </c>
-      <c r="AE184" s="14" t="inlineStr"/>
-      <c r="AF184" s="14" t="inlineStr"/>
-      <c r="AG184" s="14" t="inlineStr"/>
+      <c r="AE184" s="14" t="n">
+        <v>39008.97</v>
+      </c>
+      <c r="AF184" s="14" t="n"/>
+      <c r="AG184" s="14" t="n"/>
       <c r="AH184" s="14" t="inlineStr"/>
       <c r="AI184" s="14" t="inlineStr">
         <is>
@@ -26544,9 +26546,11 @@
       <c r="AD185" s="14" t="n">
         <v>0.9434799273257846</v>
       </c>
-      <c r="AE185" s="14" t="inlineStr"/>
-      <c r="AF185" s="14" t="inlineStr"/>
-      <c r="AG185" s="14" t="inlineStr"/>
+      <c r="AE185" s="14" t="n">
+        <v>109141.07</v>
+      </c>
+      <c r="AF185" s="14" t="n"/>
+      <c r="AG185" s="14" t="n"/>
       <c r="AH185" s="14" t="inlineStr"/>
       <c r="AI185" s="14" t="inlineStr">
         <is>
@@ -26700,9 +26704,11 @@
       <c r="AD186" s="14" t="n">
         <v>0.9015341796073471</v>
       </c>
-      <c r="AE186" s="14" t="inlineStr"/>
-      <c r="AF186" s="14" t="inlineStr"/>
-      <c r="AG186" s="14" t="inlineStr"/>
+      <c r="AE186" s="14" t="n">
+        <v>31915.58</v>
+      </c>
+      <c r="AF186" s="14" t="n"/>
+      <c r="AG186" s="14" t="n"/>
       <c r="AH186" s="14" t="inlineStr"/>
       <c r="AI186" s="14" t="inlineStr">
         <is>
@@ -26856,9 +26862,11 @@
       <c r="AD187" s="14" t="n">
         <v>0.9644186733928968</v>
       </c>
-      <c r="AE187" s="14" t="inlineStr"/>
-      <c r="AF187" s="14" t="inlineStr"/>
-      <c r="AG187" s="14" t="inlineStr"/>
+      <c r="AE187" s="14" t="n">
+        <v>11780.27</v>
+      </c>
+      <c r="AF187" s="14" t="n"/>
+      <c r="AG187" s="14" t="n"/>
       <c r="AH187" s="14" t="inlineStr"/>
       <c r="AI187" s="14" t="inlineStr">
         <is>
@@ -27012,9 +27020,11 @@
       <c r="AD188" s="14" t="n">
         <v>0.7858113084952347</v>
       </c>
-      <c r="AE188" s="14" t="inlineStr"/>
-      <c r="AF188" s="14" t="inlineStr"/>
-      <c r="AG188" s="14" t="inlineStr"/>
+      <c r="AE188" s="14" t="n">
+        <v>14750.12</v>
+      </c>
+      <c r="AF188" s="14" t="n"/>
+      <c r="AG188" s="14" t="n"/>
       <c r="AH188" s="14" t="inlineStr"/>
       <c r="AI188" s="14" t="inlineStr">
         <is>
@@ -27168,9 +27178,11 @@
       <c r="AD189" s="14" t="n">
         <v>1.132241909977781</v>
       </c>
-      <c r="AE189" s="14" t="inlineStr"/>
-      <c r="AF189" s="14" t="inlineStr"/>
-      <c r="AG189" s="14" t="inlineStr"/>
+      <c r="AE189" s="14" t="n">
+        <v>7075.24</v>
+      </c>
+      <c r="AF189" s="14" t="n"/>
+      <c r="AG189" s="14" t="n"/>
       <c r="AH189" s="14" t="inlineStr"/>
       <c r="AI189" s="14" t="inlineStr">
         <is>
@@ -27328,9 +27340,11 @@
       <c r="AD190" s="14" t="n">
         <v>0.8911750740595309</v>
       </c>
-      <c r="AE190" s="14" t="inlineStr"/>
-      <c r="AF190" s="14" t="inlineStr"/>
-      <c r="AG190" s="14" t="inlineStr"/>
+      <c r="AE190" s="14" t="n">
+        <v>25013.15</v>
+      </c>
+      <c r="AF190" s="14" t="n"/>
+      <c r="AG190" s="14" t="n"/>
       <c r="AH190" s="14" t="inlineStr"/>
       <c r="AI190" s="14" t="inlineStr">
         <is>
@@ -27484,9 +27498,11 @@
       <c r="AD191" s="14" t="n">
         <v>0.9087126489086662</v>
       </c>
-      <c r="AE191" s="14" t="inlineStr"/>
-      <c r="AF191" s="14" t="inlineStr"/>
-      <c r="AG191" s="14" t="inlineStr"/>
+      <c r="AE191" s="14" t="n">
+        <v>35631.35</v>
+      </c>
+      <c r="AF191" s="14" t="n"/>
+      <c r="AG191" s="14" t="n"/>
       <c r="AH191" s="14" t="inlineStr"/>
       <c r="AI191" s="14" t="inlineStr">
         <is>
@@ -27640,9 +27656,11 @@
       <c r="AD192" s="14" t="n">
         <v>1.0338226823344</v>
       </c>
-      <c r="AE192" s="14" t="inlineStr"/>
-      <c r="AF192" s="14" t="inlineStr"/>
-      <c r="AG192" s="14" t="inlineStr"/>
+      <c r="AE192" s="14" t="n">
+        <v>19225.53</v>
+      </c>
+      <c r="AF192" s="14" t="n"/>
+      <c r="AG192" s="14" t="n"/>
       <c r="AH192" s="14" t="inlineStr"/>
       <c r="AI192" s="14" t="inlineStr">
         <is>
@@ -27796,9 +27814,11 @@
       <c r="AD193" s="14" t="n">
         <v>0.9170282507910528</v>
       </c>
-      <c r="AE193" s="14" t="inlineStr"/>
-      <c r="AF193" s="14" t="inlineStr"/>
-      <c r="AG193" s="14" t="inlineStr"/>
+      <c r="AE193" s="14" t="n">
+        <v>52464.98</v>
+      </c>
+      <c r="AF193" s="14" t="n"/>
+      <c r="AG193" s="14" t="n"/>
       <c r="AH193" s="14" t="inlineStr"/>
       <c r="AI193" s="14" t="inlineStr">
         <is>
@@ -27952,9 +27972,11 @@
       <c r="AD194" s="14" t="n">
         <v>0.9957709450100648</v>
       </c>
-      <c r="AE194" s="14" t="inlineStr"/>
-      <c r="AF194" s="14" t="inlineStr"/>
-      <c r="AG194" s="14" t="inlineStr"/>
+      <c r="AE194" s="14" t="n">
+        <v>18217.9</v>
+      </c>
+      <c r="AF194" s="14" t="n"/>
+      <c r="AG194" s="14" t="n"/>
       <c r="AH194" s="14" t="inlineStr"/>
       <c r="AI194" s="14" t="inlineStr">
         <is>
@@ -28108,9 +28130,11 @@
       <c r="AD195" s="14" t="n">
         <v>1.109403629594396</v>
       </c>
-      <c r="AE195" s="14" t="inlineStr"/>
-      <c r="AF195" s="14" t="inlineStr"/>
-      <c r="AG195" s="14" t="inlineStr"/>
+      <c r="AE195" s="14" t="n">
+        <v>18247.36</v>
+      </c>
+      <c r="AF195" s="14" t="n"/>
+      <c r="AG195" s="14" t="n"/>
       <c r="AH195" s="14" t="inlineStr"/>
       <c r="AI195" s="14" t="inlineStr">
         <is>
@@ -28264,9 +28288,11 @@
       <c r="AD196" s="14" t="n">
         <v>1.045502810395282</v>
       </c>
-      <c r="AE196" s="14" t="inlineStr"/>
-      <c r="AF196" s="14" t="inlineStr"/>
-      <c r="AG196" s="14" t="inlineStr"/>
+      <c r="AE196" s="14" t="n">
+        <v>13740.33</v>
+      </c>
+      <c r="AF196" s="14" t="n"/>
+      <c r="AG196" s="14" t="n"/>
       <c r="AH196" s="14" t="inlineStr"/>
       <c r="AI196" s="14" t="inlineStr">
         <is>
@@ -28424,9 +28450,11 @@
       <c r="AD197" s="14" t="n">
         <v>1.206433790586367</v>
       </c>
-      <c r="AE197" s="14" t="inlineStr"/>
-      <c r="AF197" s="14" t="inlineStr"/>
-      <c r="AG197" s="14" t="inlineStr"/>
+      <c r="AE197" s="14" t="n">
+        <v>9330.370000000001</v>
+      </c>
+      <c r="AF197" s="14" t="n"/>
+      <c r="AG197" s="14" t="n"/>
       <c r="AH197" s="14" t="inlineStr"/>
       <c r="AI197" s="14" t="inlineStr">
         <is>
@@ -28580,9 +28608,11 @@
       <c r="AD198" s="14" t="n">
         <v>1.023992551469679</v>
       </c>
-      <c r="AE198" s="14" t="inlineStr"/>
-      <c r="AF198" s="14" t="inlineStr"/>
-      <c r="AG198" s="14" t="inlineStr"/>
+      <c r="AE198" s="14" t="n">
+        <v>34544.31</v>
+      </c>
+      <c r="AF198" s="14" t="n"/>
+      <c r="AG198" s="14" t="n"/>
       <c r="AH198" s="14" t="inlineStr"/>
       <c r="AI198" s="14" t="inlineStr">
         <is>
@@ -28740,9 +28770,11 @@
       <c r="AD199" s="14" t="n">
         <v>1.103748875760919</v>
       </c>
-      <c r="AE199" s="14" t="inlineStr"/>
-      <c r="AF199" s="14" t="inlineStr"/>
-      <c r="AG199" s="14" t="inlineStr"/>
+      <c r="AE199" s="14" t="n">
+        <v>7124.46</v>
+      </c>
+      <c r="AF199" s="14" t="n"/>
+      <c r="AG199" s="14" t="n"/>
       <c r="AH199" s="14" t="inlineStr"/>
       <c r="AI199" s="14" t="inlineStr">
         <is>
@@ -28900,9 +28932,11 @@
       <c r="AD200" s="14" t="n">
         <v>1.012860270317046</v>
       </c>
-      <c r="AE200" s="14" t="inlineStr"/>
-      <c r="AF200" s="14" t="inlineStr"/>
-      <c r="AG200" s="14" t="inlineStr"/>
+      <c r="AE200" s="14" t="n">
+        <v>10668.41</v>
+      </c>
+      <c r="AF200" s="14" t="n"/>
+      <c r="AG200" s="14" t="n"/>
       <c r="AH200" s="14" t="inlineStr"/>
       <c r="AI200" s="14" t="inlineStr">
         <is>
@@ -29040,9 +29074,11 @@
       <c r="AD201" s="14" t="n">
         <v>1.0609</v>
       </c>
-      <c r="AE201" s="14" t="inlineStr"/>
-      <c r="AF201" s="14" t="inlineStr"/>
-      <c r="AG201" s="14" t="inlineStr"/>
+      <c r="AE201" s="14" t="n">
+        <v>17173.18</v>
+      </c>
+      <c r="AF201" s="14" t="n"/>
+      <c r="AG201" s="14" t="n"/>
       <c r="AH201" s="14" t="inlineStr"/>
       <c r="AI201" s="14" t="inlineStr">
         <is>
@@ -29198,9 +29234,13 @@
       <c r="AD202" s="14" t="n">
         <v>0.913</v>
       </c>
-      <c r="AE202" s="14" t="inlineStr"/>
-      <c r="AF202" s="14" t="inlineStr"/>
-      <c r="AG202" s="14" t="inlineStr"/>
+      <c r="AE202" s="14" t="n">
+        <v>14686.24</v>
+      </c>
+      <c r="AF202" s="14" t="n"/>
+      <c r="AG202" s="14" t="n">
+        <v>0.003653</v>
+      </c>
       <c r="AH202" s="14" t="inlineStr"/>
       <c r="AI202" s="14" t="inlineStr">
         <is>
@@ -29356,9 +29396,13 @@
       <c r="AD203" s="14" t="n">
         <v>1.015</v>
       </c>
-      <c r="AE203" s="14" t="inlineStr"/>
-      <c r="AF203" s="14" t="inlineStr"/>
-      <c r="AG203" s="14" t="inlineStr"/>
+      <c r="AE203" s="14" t="n">
+        <v>70493.67999999999</v>
+      </c>
+      <c r="AF203" s="14" t="n"/>
+      <c r="AG203" s="14" t="n">
+        <v>0.017628</v>
+      </c>
       <c r="AH203" s="14" t="inlineStr"/>
       <c r="AI203" s="14" t="inlineStr">
         <is>
@@ -29512,9 +29556,13 @@
       <c r="AD204" s="14" t="n">
         <v>0.8641</v>
       </c>
-      <c r="AE204" s="14" t="inlineStr"/>
-      <c r="AF204" s="14" t="inlineStr"/>
-      <c r="AG204" s="14" t="inlineStr"/>
+      <c r="AE204" s="14" t="n">
+        <v>53640.77</v>
+      </c>
+      <c r="AF204" s="14" t="n"/>
+      <c r="AG204" s="14" t="n">
+        <v>0.012011</v>
+      </c>
       <c r="AH204" s="14" t="inlineStr"/>
       <c r="AI204" s="14" t="inlineStr">
         <is>
@@ -29672,9 +29720,13 @@
       <c r="AD205" s="14" t="n">
         <v>0.9496</v>
       </c>
-      <c r="AE205" s="14" t="inlineStr"/>
-      <c r="AF205" s="14" t="inlineStr"/>
-      <c r="AG205" s="14" t="inlineStr"/>
+      <c r="AE205" s="14" t="n">
+        <v>25009.93</v>
+      </c>
+      <c r="AF205" s="14" t="n"/>
+      <c r="AG205" s="14" t="n">
+        <v>0.005674</v>
+      </c>
       <c r="AH205" s="14" t="inlineStr"/>
       <c r="AI205" s="14" t="inlineStr">
         <is>
@@ -29830,9 +29882,13 @@
       <c r="AD206" s="14" t="n">
         <v>0.8852</v>
       </c>
-      <c r="AE206" s="14" t="inlineStr"/>
-      <c r="AF206" s="14" t="inlineStr"/>
-      <c r="AG206" s="14" t="inlineStr"/>
+      <c r="AE206" s="14" t="n">
+        <v>20805.3</v>
+      </c>
+      <c r="AF206" s="14" t="n"/>
+      <c r="AG206" s="14" t="n">
+        <v>0.00448</v>
+      </c>
       <c r="AH206" s="14" t="inlineStr"/>
       <c r="AI206" s="14" t="inlineStr">
         <is>
@@ -29990,9 +30046,13 @@
       <c r="AD207" s="14" t="n">
         <v>0.893</v>
       </c>
-      <c r="AE207" s="14" t="inlineStr"/>
-      <c r="AF207" s="14" t="inlineStr"/>
-      <c r="AG207" s="14" t="inlineStr"/>
+      <c r="AE207" s="14" t="n">
+        <v>11669.93</v>
+      </c>
+      <c r="AF207" s="14" t="n"/>
+      <c r="AG207" s="14" t="n">
+        <v>0.002556</v>
+      </c>
       <c r="AH207" s="14" t="inlineStr"/>
       <c r="AI207" s="14" t="inlineStr">
         <is>
@@ -30150,9 +30210,13 @@
       <c r="AD208" s="14" t="n">
         <v>1.1734</v>
       </c>
-      <c r="AE208" s="14" t="inlineStr"/>
-      <c r="AF208" s="14" t="inlineStr"/>
-      <c r="AG208" s="14" t="inlineStr"/>
+      <c r="AE208" s="14" t="n">
+        <v>8067.23</v>
+      </c>
+      <c r="AF208" s="14" t="n"/>
+      <c r="AG208" s="14" t="n">
+        <v>0.001765</v>
+      </c>
       <c r="AH208" s="14" t="inlineStr"/>
       <c r="AI208" s="14" t="inlineStr">
         <is>
@@ -30312,9 +30376,13 @@
       <c r="AD209" s="14" t="n">
         <v>0.8561</v>
       </c>
-      <c r="AE209" s="14" t="inlineStr"/>
-      <c r="AF209" s="14" t="inlineStr"/>
-      <c r="AG209" s="14" t="inlineStr"/>
+      <c r="AE209" s="14" t="n">
+        <v>24792.52</v>
+      </c>
+      <c r="AF209" s="14" t="n"/>
+      <c r="AG209" s="14" t="n">
+        <v>0.005282</v>
+      </c>
       <c r="AH209" s="14" t="inlineStr"/>
       <c r="AI209" s="14" t="inlineStr">
         <is>
@@ -30474,9 +30542,13 @@
       <c r="AD210" s="14" t="n">
         <v>0.8754999999999999</v>
       </c>
-      <c r="AE210" s="14" t="inlineStr"/>
-      <c r="AF210" s="14" t="inlineStr"/>
-      <c r="AG210" s="14" t="inlineStr"/>
+      <c r="AE210" s="14" t="n">
+        <v>41213.72</v>
+      </c>
+      <c r="AF210" s="14" t="n"/>
+      <c r="AG210" s="14" t="n">
+        <v>0.008987</v>
+      </c>
       <c r="AH210" s="14" t="inlineStr"/>
       <c r="AI210" s="14" t="inlineStr">
         <is>
@@ -30636,9 +30708,13 @@
       <c r="AD211" s="14" t="n">
         <v>1.0308</v>
       </c>
-      <c r="AE211" s="14" t="inlineStr"/>
-      <c r="AF211" s="14" t="inlineStr"/>
-      <c r="AG211" s="14" t="inlineStr"/>
+      <c r="AE211" s="14" t="n">
+        <v>20313.12</v>
+      </c>
+      <c r="AF211" s="14" t="n"/>
+      <c r="AG211" s="14" t="n">
+        <v>0.004863</v>
+      </c>
       <c r="AH211" s="14" t="inlineStr"/>
       <c r="AI211" s="14" t="inlineStr">
         <is>
@@ -30800,9 +30876,13 @@
       <c r="AD212" s="14" t="n">
         <v>0.8006</v>
       </c>
-      <c r="AE212" s="14" t="inlineStr"/>
-      <c r="AF212" s="14" t="inlineStr"/>
-      <c r="AG212" s="14" t="inlineStr"/>
+      <c r="AE212" s="14" t="n">
+        <v>12686.24</v>
+      </c>
+      <c r="AF212" s="14" t="n"/>
+      <c r="AG212" s="14" t="n">
+        <v>0.002901</v>
+      </c>
       <c r="AH212" s="14" t="inlineStr"/>
       <c r="AI212" s="14" t="inlineStr">
         <is>
@@ -30964,9 +31044,13 @@
       <c r="AD213" s="14" t="n">
         <v>1.0375</v>
       </c>
-      <c r="AE213" s="14" t="inlineStr"/>
-      <c r="AF213" s="14" t="inlineStr"/>
-      <c r="AG213" s="14" t="inlineStr"/>
+      <c r="AE213" s="14" t="n">
+        <v>60684.07</v>
+      </c>
+      <c r="AF213" s="14" t="n"/>
+      <c r="AG213" s="14" t="n">
+        <v>0.014416</v>
+      </c>
       <c r="AH213" s="14" t="inlineStr"/>
       <c r="AI213" s="14" t="inlineStr">
         <is>
@@ -31128,9 +31212,13 @@
       <c r="AD214" s="14" t="n">
         <v>1.1686</v>
       </c>
-      <c r="AE214" s="14" t="inlineStr"/>
-      <c r="AF214" s="14" t="inlineStr"/>
-      <c r="AG214" s="14" t="inlineStr"/>
+      <c r="AE214" s="14" t="n">
+        <v>34815.46</v>
+      </c>
+      <c r="AF214" s="14" t="n"/>
+      <c r="AG214" s="14" t="n">
+        <v>0.007901999999999999</v>
+      </c>
       <c r="AH214" s="14" t="inlineStr"/>
       <c r="AI214" s="14" t="inlineStr">
         <is>
@@ -31296,9 +31384,13 @@
       <c r="AD215" s="14" t="n">
         <v>0.9866</v>
       </c>
-      <c r="AE215" s="14" t="inlineStr"/>
-      <c r="AF215" s="14" t="inlineStr"/>
-      <c r="AG215" s="14" t="inlineStr"/>
+      <c r="AE215" s="14" t="n">
+        <v>13580.19</v>
+      </c>
+      <c r="AF215" s="14" t="n"/>
+      <c r="AG215" s="14" t="n">
+        <v>0.003516</v>
+      </c>
       <c r="AH215" s="14" t="inlineStr"/>
       <c r="AI215" s="14" t="inlineStr">
         <is>
@@ -31460,9 +31552,13 @@
       <c r="AD216" s="14" t="n">
         <v>0.993</v>
       </c>
-      <c r="AE216" s="14" t="inlineStr"/>
-      <c r="AF216" s="14" t="inlineStr"/>
-      <c r="AG216" s="14" t="inlineStr"/>
+      <c r="AE216" s="14" t="n">
+        <v>24051.96</v>
+      </c>
+      <c r="AF216" s="14" t="n"/>
+      <c r="AG216" s="14" t="n">
+        <v>0.005826</v>
+      </c>
       <c r="AH216" s="14" t="inlineStr"/>
       <c r="AI216" s="14" t="inlineStr">
         <is>
@@ -31624,9 +31720,13 @@
       <c r="AD217" s="14" t="n">
         <v>1.0262</v>
       </c>
-      <c r="AE217" s="14" t="inlineStr"/>
-      <c r="AF217" s="14" t="inlineStr"/>
-      <c r="AG217" s="14" t="inlineStr"/>
+      <c r="AE217" s="14" t="n">
+        <v>22806.38</v>
+      </c>
+      <c r="AF217" s="14" t="n"/>
+      <c r="AG217" s="14" t="n">
+        <v>0.005539</v>
+      </c>
       <c r="AH217" s="14" t="inlineStr"/>
       <c r="AI217" s="14" t="inlineStr">
         <is>
@@ -31792,9 +31892,13 @@
       <c r="AD218" s="14" t="n">
         <v>0.9176</v>
       </c>
-      <c r="AE218" s="14" t="inlineStr"/>
-      <c r="AF218" s="14" t="inlineStr"/>
-      <c r="AG218" s="14" t="inlineStr"/>
+      <c r="AE218" s="14" t="n">
+        <v>16948.18</v>
+      </c>
+      <c r="AF218" s="14" t="n"/>
+      <c r="AG218" s="14" t="n">
+        <v>0.0043</v>
+      </c>
       <c r="AH218" s="14" t="inlineStr"/>
       <c r="AI218" s="14" t="inlineStr">
         <is>
@@ -31956,9 +32060,13 @@
       <c r="AD219" s="14" t="n">
         <v>0.7741</v>
       </c>
-      <c r="AE219" s="14" t="inlineStr"/>
-      <c r="AF219" s="14" t="inlineStr"/>
-      <c r="AG219" s="14" t="inlineStr"/>
+      <c r="AE219" s="14" t="n">
+        <v>34468.24</v>
+      </c>
+      <c r="AF219" s="14" t="n"/>
+      <c r="AG219" s="14" t="n">
+        <v>0.008938</v>
+      </c>
       <c r="AH219" s="14" t="inlineStr"/>
       <c r="AI219" s="14" t="inlineStr">
         <is>
@@ -32120,9 +32228,13 @@
       <c r="AD220" s="14" t="n">
         <v>0.9661999999999999</v>
       </c>
-      <c r="AE220" s="14" t="inlineStr"/>
-      <c r="AF220" s="14" t="inlineStr"/>
-      <c r="AG220" s="14" t="inlineStr"/>
+      <c r="AE220" s="14" t="n">
+        <v>37284.79</v>
+      </c>
+      <c r="AF220" s="14" t="n"/>
+      <c r="AG220" s="14" t="n">
+        <v>0.009745</v>
+      </c>
       <c r="AH220" s="14" t="inlineStr"/>
       <c r="AI220" s="14" t="inlineStr">
         <is>
@@ -32284,9 +32396,13 @@
       <c r="AD221" s="14" t="n">
         <v>0.8985</v>
       </c>
-      <c r="AE221" s="14" t="inlineStr"/>
-      <c r="AF221" s="14" t="inlineStr"/>
-      <c r="AG221" s="14" t="inlineStr"/>
+      <c r="AE221" s="14" t="n">
+        <v>32962.78</v>
+      </c>
+      <c r="AF221" s="14" t="n"/>
+      <c r="AG221" s="14" t="n">
+        <v>0.008376</v>
+      </c>
       <c r="AH221" s="14" t="inlineStr"/>
       <c r="AI221" s="14" t="inlineStr">
         <is>
@@ -32448,9 +32564,13 @@
       <c r="AD222" s="14" t="n">
         <v>0.9351</v>
       </c>
-      <c r="AE222" s="14" t="inlineStr"/>
-      <c r="AF222" s="14" t="inlineStr"/>
-      <c r="AG222" s="14" t="inlineStr"/>
+      <c r="AE222" s="14" t="n">
+        <v>19267.37</v>
+      </c>
+      <c r="AF222" s="14" t="n"/>
+      <c r="AG222" s="14" t="n">
+        <v>0.004368</v>
+      </c>
       <c r="AH222" s="14" t="inlineStr"/>
       <c r="AI222" s="14" t="inlineStr">
         <is>
@@ -32612,9 +32732,13 @@
       <c r="AD223" s="14" t="n">
         <v>0.8406</v>
       </c>
-      <c r="AE223" s="14" t="inlineStr"/>
-      <c r="AF223" s="14" t="inlineStr"/>
-      <c r="AG223" s="14" t="inlineStr"/>
+      <c r="AE223" s="14" t="n">
+        <v>44443.64</v>
+      </c>
+      <c r="AF223" s="14" t="n"/>
+      <c r="AG223" s="14" t="n">
+        <v>0.010123</v>
+      </c>
       <c r="AH223" s="14" t="inlineStr"/>
       <c r="AI223" s="14" t="inlineStr">
         <is>
@@ -32776,9 +32900,13 @@
       <c r="AD224" s="14" t="n">
         <v>0.9691</v>
       </c>
-      <c r="AE224" s="14" t="inlineStr"/>
-      <c r="AF224" s="14" t="inlineStr"/>
-      <c r="AG224" s="14" t="inlineStr"/>
+      <c r="AE224" s="14" t="n">
+        <v>11388.28</v>
+      </c>
+      <c r="AF224" s="14" t="n"/>
+      <c r="AG224" s="14" t="n">
+        <v>0.00273</v>
+      </c>
       <c r="AH224" s="14" t="inlineStr"/>
       <c r="AI224" s="14" t="inlineStr">
         <is>
@@ -32940,9 +33068,13 @@
       <c r="AD225" s="14" t="n">
         <v>0.9184</v>
       </c>
-      <c r="AE225" s="14" t="inlineStr"/>
-      <c r="AF225" s="14" t="inlineStr"/>
-      <c r="AG225" s="14" t="inlineStr"/>
+      <c r="AE225" s="14" t="n">
+        <v>20485.49</v>
+      </c>
+      <c r="AF225" s="14" t="n"/>
+      <c r="AG225" s="14" t="n">
+        <v>0.004977</v>
+      </c>
       <c r="AH225" s="14" t="inlineStr"/>
       <c r="AI225" s="14" t="inlineStr">
         <is>
@@ -33104,9 +33236,13 @@
       <c r="AD226" s="14" t="n">
         <v>0.9389999999999999</v>
       </c>
-      <c r="AE226" s="14" t="inlineStr"/>
-      <c r="AF226" s="14" t="inlineStr"/>
-      <c r="AG226" s="14" t="inlineStr"/>
+      <c r="AE226" s="14" t="n">
+        <v>22964.8</v>
+      </c>
+      <c r="AF226" s="14" t="n"/>
+      <c r="AG226" s="14" t="n">
+        <v>0.005033</v>
+      </c>
       <c r="AH226" s="14" t="inlineStr"/>
       <c r="AI226" s="14" t="inlineStr">
         <is>
@@ -33268,9 +33404,13 @@
       <c r="AD227" s="14" t="n">
         <v>0.9887</v>
       </c>
-      <c r="AE227" s="14" t="inlineStr"/>
-      <c r="AF227" s="14" t="inlineStr"/>
-      <c r="AG227" s="14" t="inlineStr"/>
+      <c r="AE227" s="14" t="n">
+        <v>41492.27</v>
+      </c>
+      <c r="AF227" s="14" t="n"/>
+      <c r="AG227" s="14" t="n">
+        <v>0.009398</v>
+      </c>
       <c r="AH227" s="14" t="inlineStr"/>
       <c r="AI227" s="14" t="inlineStr">
         <is>
@@ -33432,9 +33572,13 @@
       <c r="AD228" s="14" t="n">
         <v>0.8907</v>
       </c>
-      <c r="AE228" s="14" t="inlineStr"/>
-      <c r="AF228" s="14" t="inlineStr"/>
-      <c r="AG228" s="14" t="inlineStr"/>
+      <c r="AE228" s="14" t="n">
+        <v>46055.74</v>
+      </c>
+      <c r="AF228" s="14" t="n"/>
+      <c r="AG228" s="14" t="n">
+        <v>0.009702000000000001</v>
+      </c>
       <c r="AH228" s="14" t="inlineStr"/>
       <c r="AI228" s="14" t="inlineStr">
         <is>
@@ -33596,9 +33740,13 @@
       <c r="AD229" s="14" t="n">
         <v>0.8709</v>
       </c>
-      <c r="AE229" s="14" t="inlineStr"/>
-      <c r="AF229" s="14" t="inlineStr"/>
-      <c r="AG229" s="14" t="inlineStr"/>
+      <c r="AE229" s="14" t="n">
+        <v>60038.13</v>
+      </c>
+      <c r="AF229" s="14" t="n"/>
+      <c r="AG229" s="14" t="n">
+        <v>0.012707</v>
+      </c>
       <c r="AH229" s="14" t="inlineStr"/>
       <c r="AI229" s="14" t="inlineStr">
         <is>
@@ -33760,9 +33908,13 @@
       <c r="AD230" s="14" t="n">
         <v>0.8319</v>
       </c>
-      <c r="AE230" s="14" t="inlineStr"/>
-      <c r="AF230" s="14" t="inlineStr"/>
-      <c r="AG230" s="14" t="inlineStr"/>
+      <c r="AE230" s="14" t="n">
+        <v>10664.35</v>
+      </c>
+      <c r="AF230" s="14" t="n"/>
+      <c r="AG230" s="14" t="n">
+        <v>0.002228</v>
+      </c>
       <c r="AH230" s="14" t="inlineStr"/>
       <c r="AI230" s="14" t="inlineStr">
         <is>

</xml_diff>